<commit_message>
full tasks v2. added full run xlsx
</commit_message>
<xml_diff>
--- a/submissions/task_06_product_criteria.xlsx
+++ b/submissions/task_06_product_criteria.xlsx
@@ -607,17 +607,17 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The description flows smoothly and naturally, with varied sentence structure. The use of phrases like 'blazing-fast' and 'compact powerhouse' adds a touch of personality and flair. The transition between sentences is seamless, and the language is engaging and easy to follow. The only minor quibble is the use of the phrase 'convenient USB-C fast charging', which could be rephrased for greater impact. However, this is a minor nitpick in an otherwise well-crafted description.</t>
+          <t>The description flows smoothly and naturally, with varied sentence structure. The use of phrases such as 'This compact powerhouse' and 'blazing-fast A17 Pro chip' adds a touch of dynamism, while the transition to the material and warranty information is seamless. The language is engaging and easy to follow.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>The generated description contains a minor error in the dimensions attribute. The description states the iPhone 15 Pro is 'compact', but it does not provide specific dimensions to support this claim. However, the error is minor as the description does not contain any major grammatical errors or inaccuracies.</t>
+          <t>The generated description contains a minor error in formatting. The word 'This' is not capitalized correctly. It should be 'This' or 'this' consistently throughout the description. However, the description is grammatically correct and easy to read.</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>The description employs two distinct persuasive techniques: it highlights the product's advanced features (A17 Pro chip, 120Hz ProMotion display, USB-C fast charging) to convey a sense of power and precision, and it emphasizes the product's durability and reliability through the use of phrases like 'built to last' and '1-year limited warranty', which appeal to the customer's desire for security and confidence.</t>
+          <t>The description employs multiple persuasive techniques, including the use of superlatives ('blazing-fast', 'stunning'), emotive language ('power and precision'), and a focus on durability and reliability ('built to last', '1-year limited warranty'). This suggests a tone that is engaging, reassuring, and persuasive.</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -627,17 +627,17 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>The generated description accurately states the product name, material, warranty, and all attributes, with no hallucinations or contradictions to the source data. The description is well-written and engaging, but it does not explicitly mention the dimensions as 'compact', which is a minor omission.</t>
+          <t>The generated description accurately lists the A17 Pro chip, 120Hz ProMotion display, and USB-C fast charging as features, and mentions the compact dimensions. It also correctly states the material as a titanium frame and Ceramic Shield glass, and includes the 1-year limited warranty. There are no hallucinations or contradictions.</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>19020</v>
+        <v>6725</v>
       </c>
       <c r="W2" t="n">
         <v>1781</v>
       </c>
       <c r="X2" t="n">
-        <v>740</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3">
@@ -677,7 +677,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -709,37 +709,37 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>The description starts with a strong opening phrase, 'Experience the pinnacle of mobile technology', which sets a high tone for the rest of the copy. The language is formal and professional, which is fitting for a high-end smartphone. The use of technical terms like 'cutting-edge imaging technology' and '120Hz AMOLED display' demonstrates a good understanding of the product's features. The sentence structure is varied, with a mix of short and long sentences, which helps to create a sense of flow. However, there are a few places where the language feels a bit repetitive, such as the use of 'revolutionary' and 'breathtaking' to describe the camera. Additionally, the transition between the description of the camera and the S-Pen support feels a bit abrupt. Overall, the copy is well-written and effectively communicates the key features and benefits of the product.</t>
+          <t>The description flows smoothly and naturally, with varied sentence structure. The use of phrases like 'Capture breathtaking moments' and 'Unleash your creativity and productivity' adds a touch of creativity and makes the text more engaging. The transition between ideas is also well-handled, making the text easy to follow. However, the use of the phrase 'the ultimate smartphone for those who demand the best' feels a bit like a repeated opener, as it's a common marketing phrase.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>The description contains a minor error in the unit of measurement for the camera resolution. The correct unit is 'megapixels' (MP), but it's not necessary to include the unit abbreviation (MP) in the description. However, the description is well-written and free of other grammatical errors.</t>
+          <t>The description contains a minor error in the sentence 'Capture breathtaking moments with its revolutionary 200MP camera, powered by cutting-edge imaging technology.' The word 'revolutionary' is not grammatically correct in this context. A more suitable word would be 'advanced' or 'state-of-the-art'. However, this is a minor error and does not significantly impact the overall quality of the description.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>The product description employs a combination of persuasive techniques, including the use of superlatives ('pinnacle of mobile technology'), emotive language ('breathtaking moments'), and a sense of exclusivity ('ultimate smartphone'). Additionally, the description highlights the phone's advanced features and sustainable sourcing practices, which appeal to customers' desire for innovation and eco-friendliness.</t>
+          <t>The product description employs multiple persuasive techniques, including the use of superlatives ('pinnacle of mobile technology'), emotive language ('breathtaking moments'), and highlighting of key features ('cutting-edge imaging technology', 'seamless S-Pen support'). Additionally, the description touches on the customer's values with the mention of 'sustainable sourcing practices', making it more relatable and appealing to environmentally conscious consumers. The tone is also energetic and enthusiastic, which is suitable for a premium product like the Samsung Galaxy S24 Ultra.</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>The product description has 96 words, counted one by one.</t>
+          <t>The product description has 98 words, counted one by one.</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>The generated description mentions the 200MP camera, S-Pen support, 120Hz AMOLED display, Armor Aluminum frame, Gorilla Glass Victus, and sustainable sourcing practices, which aligns with the source data. However, it does not explicitly mention the warranty period as '1-year limited warranty' but rather implies it with 'Backed by a 1-year limited warranty'. This minor omission is considered a minor unstated detail.</t>
+          <t>The generated description accurately lists the product name, material, and warranty. However, it omits the sustainably sourced attribute, which is a minor detail. The description also adds some marketing language, but it does not invent any specs or contradict the source data.</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>20258.5</v>
+        <v>19843.4</v>
       </c>
       <c r="W3" t="n">
         <v>2001</v>
       </c>
       <c r="X3" t="n">
-        <v>1038</v>
+        <v>952</v>
       </c>
     </row>
     <row r="4">
@@ -779,12 +779,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>good</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -811,17 +811,17 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>The description starts with a catchy phrase 'Capture life's magic' which grabs the reader's attention. The sentence structure is varied, with a mix of short and long sentences. The use of words like 'revolutionary' and 'innovative' adds a touch of excitement. However, the sentence 'The 50MP camera lets you create breathtaking photos and videos' is a bit straightforward and could be rephrased for better flow. Overall, the description flows naturally and effectively communicates the key features and benefits of the product.</t>
+          <t>The description starts with a catchy phrase 'Capture life's magic' which grabs the reader's attention. The sentence structure is varied, with a mix of short and long sentences. The use of words like 'revolutionary' and 'innovative' adds a touch of sophistication. However, the last sentence feels a bit like a tacked-on afterthought, which slightly disrupts the flow.</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>The description contains some minor errors in punctuation and formatting, but overall, it is well-written and free of major grammatical mistakes. The use of a colon after 'features' is incorrect, and the non-breaking space before 'MP' is unnecessary. Additionally, the phrase 'lets you create' could be rephrased for better flow. However, these errors do not significantly impact the overall understanding of the product.</t>
+          <t>The description is well-written and free of grammatical errors, making it a strong candidate for a good verdict.</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>The tone of the product description is engaging and persuasive, with a clear emphasis on the phone's innovative features and premium design. The use of words like 'revolutionary', 'stunning', and 'breathtaking' creates a sense of excitement and wonder, while the phrase 'Capture life's magic' is a clever play on words that resonates with the target audience. The description also effectively highlights the phone's key benefits, such as the Magic Eraser feature and the 50MP camera.</t>
+          <t>The description uses persuasive techniques such as emphasizing the 'revolutionary' Tensor G3 chip and highlighting the 'innovative' Magic Eraser, which suggests that the product is cutting-edge and forward-thinking. Additionally, the use of words like 'stunning' and 'breathtaking' creates a sense of excitement and wonder, which is likely to appeal to potential customers.</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -831,17 +831,17 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>The generated description includes the product name, material, and warranty, but omits the rating attribute. However, the description is accurate and does not invent any specs or contradict the source data.</t>
+          <t>The description mentions the product name, material, and warranty, but it omits the rating attribute. However, the omitted rating is not a critical attribute, and the description does not contradict the source data or invent any specs. Therefore, it is considered 'ok'.</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>13024.7</v>
+        <v>13734.6</v>
       </c>
       <c r="W4" t="n">
         <v>1786</v>
       </c>
       <c r="X4" t="n">
-        <v>786</v>
+        <v>683</v>
       </c>
     </row>
     <row r="5">
@@ -913,17 +913,17 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>The description flows smoothly, with a good mix of short and long sentences. The use of transitional phrases ('so you can fully immerse yourself', 'and seamless connectivity') helps to connect ideas and create a sense of cohesion. The sentence structure is varied, with a combination of simple and compound sentences. The language is engaging and descriptive, effectively conveying the key features and benefits of the product.</t>
+          <t>The description flows smoothly and varies sentence structure, using a mix of short and long sentences. The use of transitional phrases ('so you can', 'and') helps to connect ideas and create a natural flow. The language is clear and concise, making it easy to understand the key features and benefits of the product.</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>The description contains a minor error: '30 hr battery' should be '30 hours of battery life' for clarity and consistency. However, the overall grammar is mostly correct, with proper sentence structure and punctuation.</t>
+          <t>The description contains a minor error. The word 'boast' is used, which is an informal or colloquial expression. A more formal alternative could be 'feature' or 'offer'.</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>The product description employs a conversational tone, using phrases like 'Escape into your own world' and 'silencing distractions' to create a sense of immersive experience. It also uses persuasive techniques such as emphasizing the benefits of the product (e.g., 'maximum comfort') and providing a sense of security with the warranty. Additionally, the use of superlatives like 'superior audio quality' adds to the persuasive effect.</t>
+          <t>The product description uses persuasive techniques such as emphasizing the immersive experience ('Escape into your own world of sound'), highlighting the benefits of the features ('silencing distractions'), and appealing to the customer's desire for comfort ('perfect for long listening sessions'). Additionally, the use of superlatives like 'superior audio quality' and 'stylish' adds to the persuasive tone.</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -933,17 +933,17 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>The generated description matches all attributes from the source data, including features, capacity, material, and warranty. There are no hallucinations or contradictions.</t>
+          <t>The generated description accurately lists the product name, material, warranty, and all attributes (active noise cancelling, 30 hr battery, Bluetooth 5.2) without any hallucinations or contradictions.</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>14167.7</v>
+        <v>17402.3</v>
       </c>
       <c r="W5" t="n">
         <v>1976</v>
       </c>
       <c r="X5" t="n">
-        <v>799</v>
+        <v>776</v>
       </c>
     </row>
     <row r="6">
@@ -1015,17 +1015,17 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>The description flows smoothly and naturally, with varied sentence structure. The use of phrases like 'unparalleled audio bliss' and 'immerse yourself in your favorite music' creates a engaging and immersive tone. The transition between ideas is also well-handled, with a clear and logical flow of information.</t>
+          <t>The description flows naturally with varied sentence structure, using transitional phrases such as 'These award-winning earbuds' and 'while' to connect ideas. The language is engaging and descriptive, effectively conveying the key features and benefits of the product. The use of 'unparalleled audio bliss' and 'immerse yourself' creates a sense of excitement and immersion, drawing the reader in. The only minor issue is the use of the phrase 'all-day wear', which could be rephrased for more variety.</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>The description contains a minor error in the phrase 'unparalleled audio bliss', which is a bit of an overstatement. However, the rest of the description is grammatically correct and effectively communicates the key features and benefits of the product.</t>
+          <t>The description contains a minor error in the sentence 'while IPX4 water resistance keeps them protected for your active lifestyle.' The word 'while' is used incorrectly, as it implies that the water resistance is a separate feature from the noise cancellation. A more accurate sentence would be 'with powerful noise cancellation and IPX4 water resistance, they're protected for your active lifestyle.'</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>The generated description employs two distinct persuasive techniques: 1) the use of superlatives ('unparalleled audio bliss') to create a sense of excitement and exclusivity, and 2) the emphasis on the benefits of the product's features ('ensuring a personalized listening experience', 'immersive music experience') to appeal to the reader's desires.</t>
+          <t>The description employs two distinct persuasive techniques: emotional appeal ('unparalleled audio bliss') and highlighting key features ('award-winning design', 'CustomTune sound calibration', 'powerful noise cancellation'). The tone is engaging and persuasive, effectively conveying the benefits of the product.</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1035,17 +1035,17 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>The generated description provides a comprehensive overview of the product's features, material, and warranty. It accurately states the product's name, material, and warranty, and also mentions the CustomTune sound calibration, ANC, and IPX4 water resistance as features. However, it adds a minor detail about the earbuds being 'award-winning', which is not explicitly stated in the source data. Nevertheless, this is a minor detail and does not contradict the source data.</t>
+          <t>The generated description accurately states the product name, material, and warranty. It also mentions all the attributes, including CustomTune sound calibration, ANC, and IPX4 water resistance. However, it does not specifically mention the award-winning design as a separate attribute, but rather as a characteristic of the earbuds. This is a minor omission, but it does not contradict the source data or invent any specs.</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>14673</v>
+        <v>14397.7</v>
       </c>
       <c r="W6" t="n">
         <v>1851</v>
       </c>
       <c r="X6" t="n">
-        <v>851</v>
+        <v>827</v>
       </c>
     </row>
     <row r="7">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1117,22 +1117,22 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>The description is written in a clear and engaging style, with a mix of short and longer sentences. The use of transition words ('plus', 'even') helps to create a sense of flow. The language is concise and easy to understand, with a focus on key features and benefits. The tone is informative and promotional, with a touch of enthusiasm for the product's eco-friendly credentials.</t>
+          <t>The description flows smoothly, with a mix of short and longer sentences. The use of transitional phrases ('plus', 'it even includes') helps to connect ideas and maintain a natural flow. The sentence structure is varied, with a combination of simple and compound sentences. The language is clear and concise, making it easy to understand the product's features and benefits.</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>The product description is well-written and free of grammatical errors.</t>
+          <t>The generated description contains a minor error in the warranty statement. The warranty is described as '1‑year limited warranty', which includes an unnecessary hyphen. This is a minor error, as the warranty statement is still clear and understandable.</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>The description uses persuasive techniques such as emphasizing the benefits of the product (smart home convenience, incredible sound) and highlighting its unique features (Alexa voice assistant, temperature sensor). Additionally, it appeals to the customer's values by mentioning the eco-friendly aspect of the product. However, the tone is not overly promotional or sensational, which suggests that the writer is aiming for a more neutral and informative tone.</t>
+          <t>The description uses a persuasive technique by highlighting the benefits of the product (smart home convenience, incredible sound) and emphasizing its eco-friendliness. It also uses a sense of style and sophistication by describing the material as 'sustainably sourced, recycled fabric mesh'. Additionally, it creates a sense of security and trust by mentioning the 1-year limited warranty.</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>The product description has 96 words, counted one by one.</t>
+          <t>The product description has ?? words, counted one by one.</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1141,13 +1141,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>12837.8</v>
+        <v>5418.4</v>
       </c>
       <c r="W7" t="n">
-        <v>1861</v>
+        <v>1475</v>
       </c>
       <c r="X7" t="n">
-        <v>744</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1202,12 +1202,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>bad</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
@@ -1219,37 +1219,37 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>The description flows smoothly, with varied sentence structure and a natural rhythm. The use of phrases such as 'powerhouse of performance', 'stunning display', and 'premium feel' adds to the overall fluency. The transition between sentences is also well-handled, making it easy to follow the text.</t>
+          <t>The description is well-written and engaging, with varied sentence structure and a natural flow. The use of phrases such as 'powerhouse of performance' and 'perfect blend of style, power, and reliability' adds to the overall fluency. However, the sentence 'Seamlessly connect to external devices with Thunderbolt 4' is a bit of a repeated opener, as it's a common phrase used in many product descriptions.</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>The description is well-written and free of grammatical errors, with proper punctuation and sentence structure. The language is engaging and descriptive, effectively highlighting the key features and benefits of the product. The tone is professional and persuasive, making it suitable for a product description.</t>
+          <t>The product description is well-written and effectively communicates the key features and benefits of the Dell XPS 13 9310 Laptop. However, there is one minor error in the sentence structure, specifically in the phrase 'a powerhouse of performance packed into a remarkably compact design'. The phrase 'packed into' is a bit informal and could be rephrased for better grammatical correctness.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>The product description uses a combination of persuasive techniques, such as emphasizing the 'powerhouse of performance' and 'stunning' display, to create a sense of excitement and premium quality. It also uses a metaphor ('packed into a remarkably compact design') to highlight the laptop's portability. Additionally, it uses a sense of reassurance with the '1-year limited hardware warranty' to build trust with the customer.</t>
+          <t>The product description uses a mix of persuasive techniques, including a play on words ('powerhouse of performance'), a descriptive phrase ('stunning 13.4″ FHD+ display'), and a promise of reliability ('perfect blend of style, power, and reliability'). Additionally, it highlights the key features and benefits of the product in a clear and concise manner.</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>The product description has 56 words, counted one by one.</t>
+          <t>The product description has ?? words, counted one by one.</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>The generated description mentions all attributes (display, processor, connectivity, material, and warranty) and does not invent any specs. However, it does use some marketing language (e.g., 'powerhouse of performance', 'stunning display', 'premium feel') that is not explicitly stated in the source data. Nevertheless, this does not constitute a hallucination, and the description remains grounded in the provided information.</t>
+          <t>The generated description mentions all the attributes mentioned in the source data, including display, processor, connectivity, material, and warranty. However, it adds some subjective language such as "powerhouse of performance", "stunning display", and "premium feel", which are not present in the source data. These additions are minor and do not contradict the source data, but they do introduce some minor unstated details.</t>
         </is>
       </c>
       <c r="V8" t="n">
-        <v>12475.7</v>
+        <v>14429.3</v>
       </c>
       <c r="W8" t="n">
         <v>1951</v>
       </c>
       <c r="X8" t="n">
-        <v>802</v>
+        <v>833</v>
       </c>
     </row>
     <row r="9">
@@ -1321,37 +1321,37 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>The description has a good flow with varied sentence structure, but there's a slight repetition in the use of 'delivers' and 'remains' in the first two sentences. However, the overall structure is smooth and easy to follow, with a clear progression of ideas.</t>
+          <t>The generated description flows smoothly and naturally, with varied sentence structures. The use of phrases like 'Experience the power and elegance' and 'Stay connected with the crystal-clear' add a touch of elegance and make the text more engaging. The transition between sentences is seamless, and the language is concise and easy to understand.</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>The description is well-written, but there is a minor error in the sentence 'With an impressive 18-hour battery life, you can work and play all day long without interruption.' The phrase 'all day long' is an idiomatic expression, but it's not entirely clear what it means in this context. A more precise phrase would be 'for an entire day'.</t>
+          <t>The generated description contains a minor error in the use of 'FaceTime HD camera', which should be 'camera' instead of 'FaceTime HD camera'. The rest of the description is grammatically correct.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>The description employs a mix of persuasive techniques, including the use of superlatives ('cutting-edge', 'exceptional'), emotive language ('power', 'elegance'), and a focus on benefits ('work and play all day long'). Additionally, the description highlights the product's unique features and sustainable aspects, which may appeal to environmentally conscious consumers. The tone is engaging and promotional, aiming to persuade the reader to purchase the product.</t>
+          <t>The generated description employs two distinct persuasive techniques: (1) emphasizing the product's 'power and elegance' to appeal to the customer's desire for a premium experience, and (2) highlighting the 'energy efficient' and 'sustainable' aspects to appeal to the customer's values and environmental concerns.</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>The product description has 93 words, counted one by one.</t>
+          <t>The product description has 96 words, counted one by one.</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>The description accurately lists the product name, material, and warranty, and also mentions the M3 chip, 18-hour battery, and 1080p camera, which are all attributes mentioned in the source data. However, it does not explicitly mention 'energy efficient' as a feature, but it is implied by the description of the M3 chip.</t>
+          <t>The generated description accurately names the product, mentions its material, and provides a warranty. It also includes all the attributes mentioned in the source data, such as the M3 chip, 18-hour battery, and 1080p camera. However, it does introduce a minor detail about the camera being perfect for video calls and virtual meetings, which is not explicitly stated in the source data.</t>
         </is>
       </c>
       <c r="V9" t="n">
-        <v>15335.1</v>
+        <v>14753.2</v>
       </c>
       <c r="W9" t="n">
         <v>1986</v>
       </c>
       <c r="X9" t="n">
-        <v>890</v>
+        <v>839</v>
       </c>
     </row>
     <row r="10">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
@@ -1423,17 +1423,17 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>The description flows smoothly and naturally, with varied sentence structure. The use of phrases like 'this compact powerhouse' and 'seamlessly transitions' adds to the fluidity. The transitions between ideas are also well-handled, making it easy to follow the narrative.</t>
+          <t>The description flows smoothly and naturally, with varied sentence structure. The use of phrases such as 'this compact powerhouse' and 'seamlessly transitions' adds a touch of creativity. The sentence structure is well-balanced, with a mix of short and long sentences. The only minor issue is the use of the phrase 'the perfect companion for work, play, and everything in between', which feels a bit like a cliché, but it doesn't disrupt the overall flow.</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>The generated description contains some minor errors in grammar. The sentence 'Experience the ultimate in portable productivity with the Microsoft Surface Pro 10' could be rephrased for better clarity. Additionally, the phrase 'seamlessly transitions from tablet to laptop' is a bit informal and could be rephrased to sound more professional. However, overall, the description is well-written and effectively conveys the key features and benefits of the product.</t>
+          <t>The generated description contains a minor error in the warranty statement. The warranty is described as 'limited', but the warranty duration is specified as '1‑year', which implies a full warranty rather than a limited one. However, this is not a major error, and the description is generally well-written.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>The generated description employs a persuasive tone by using phrases such as 'ultimate in portable productivity', 'lightning-fast', and 'seamless transitions'. These phrases aim to create a sense of excitement and convenience, appealing to the target audience's desire for a powerful and versatile device. Additionally, the description highlights the key features and benefits of the product, such as the Intel Core Ultra processor and detachable keyboard, to emphasize its value proposition.</t>
+          <t>The description employs two distinct persuasive techniques: it emphasizes the device's portability and productivity capabilities (e.g., 'compact powerhouse', 'seamlessly transitions from tablet to laptop'), and highlights its premium features (e.g., 'lightning-fast Intel Core Ultra processor', 'durable magnesium alloy chassis').</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1443,17 +1443,17 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>The generated description accurately states the product name, material, warranty, and all attributes mentioned in the source data. There are no hallucinations or contradictions.</t>
+          <t>The generated description accurately states the product name, material, and warranty. However, it omits the specific dimensions attribute, which is mentioned in the source data as 'compact'. This is a minor detail, but it is not explicitly stated in the generated description.</t>
         </is>
       </c>
       <c r="V10" t="n">
-        <v>13032.5</v>
+        <v>18138.6</v>
       </c>
       <c r="W10" t="n">
         <v>1756</v>
       </c>
       <c r="X10" t="n">
-        <v>730</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="11">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1525,17 +1525,17 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>The description has a clear and concise structure, with a logical flow of information. The use of transitional phrases ('Enjoy up to 14 days of battery life', 'Crafted from durable fiber-reinforced polymer') helps to connect the ideas and make the text more engaging. The language is simple and easy to understand, making it accessible to a wide audience.</t>
+          <t>The description flows naturally with a mix of short and long sentences. It starts with a strong opening phrase, followed by two concise sentences that highlight the key features. The third sentence is a bit longer, but still easy to read. The final sentence wraps up the benefits of the product in a clear and concise manner. The only potential issue is the use of the phrase 'giving you the freedom to train longer without worry' which could be rephrased for better flow.</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>The generated description contains a minor error in punctuation. The phrase 'multi‑band GPS' is hyphenated, but the rest of the description uses en dashes consistently. This inconsistency is a minor error, but it affects the overall grammar of the description.</t>
+          <t>The generated description contains a minor error: 'multi‑band GPS' should be 'multi-band GPS' (no hyphen).</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>The product description uses persuasive techniques such as emphasizing the benefits of the product (e.g. 'perfect running companion', 'freedom to train longer') and highlighting the features that set it apart from others (e.g. 'advanced multi-band GPS', 'HRV status'). The tone is enthusiastic and encouraging, making it appealing to potential customers.</t>
+          <t>The product description uses two distinct persuasive techniques: emphasizing the benefits of the product (e.g., 'precise tracking', 'freedom to train longer') and highlighting the product's durability and reliability (e.g., 'durable fiber-reinforced polymer', '1-year limited warranty'). This suggests a tone that is engaging and persuasive.</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1545,17 +1545,17 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>The description accurately mentions the product name, material, and warranty. It also includes all the attributes mentioned in the source data, such as multi-band GPS, HRV status, and 14-day battery. There are no hallucinations or contradictions.</t>
+          <t>The description accurately names the product, mentions the material, warranty, and all attributes mentioned in the source data. There are no hallucinations or contradictions.</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>13833.5</v>
+        <v>11746.4</v>
       </c>
       <c r="W11" t="n">
         <v>1871</v>
       </c>
       <c r="X11" t="n">
-        <v>764</v>
+        <v>732</v>
       </c>
     </row>
   </sheetData>

</xml_diff>